<commit_message>
added expenditure, forms, rules, pfms, publications and UI fixes
</commit_message>
<xml_diff>
--- a/budget_documents/financialyear.xlsx
+++ b/budget_documents/financialyear.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hazel\Downloads\Delete\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DBIM Template\dbim-template\budget_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C08A62-A4B2-460B-A4B8-AABEB8E4DBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9075" yWindow="3630" windowWidth="19440" windowHeight="15600"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -19,19 +20,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Financial Year</t>
   </si>
@@ -52,12 +46,15 @@
   </si>
   <si>
     <t>2025-2026</t>
+  </si>
+  <si>
+    <t>2026-2027</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -402,45 +399,50 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added notifications and archived notifications
</commit_message>
<xml_diff>
--- a/budget_documents/financialyear.xlsx
+++ b/budget_documents/financialyear.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DBIM Template\dbim-template\budget_documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DBIM Template\budget_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2C08A62-A4B2-460B-A4B8-AABEB8E4DBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="21795" windowHeight="12975"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Financial Year</t>
   </si>
@@ -46,15 +45,12 @@
   </si>
   <si>
     <t>2025-2026</t>
-  </si>
-  <si>
-    <t>2026-2027</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -399,50 +395,45 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.45">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.45">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>